<commit_message>
İki formun iç belge numarası dosya koduyla eşitlendi; belge senkron raporu ve içerik kontrolü notu
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6foNXTwf1dGzDjULYpfrk
</commit_message>
<xml_diff>
--- a/formlar/4. Dikimhane Bölümü/EMS.QA.FRM.03.05. QA_Baskı Nakış Onay Formu.xlsx
+++ b/formlar/4. Dikimhane Bölümü/EMS.QA.FRM.03.05. QA_Baskı Nakış Onay Formu.xlsx
@@ -4897,8 +4897,10 @@
       <c r="AN2" s="87"/>
       <c r="AO2" s="87"/>
       <c r="AP2" s="87"/>
-      <c r="AQ2" s="24" t="s">
-        <v>46</v>
+      <c r="AQ2" s="24" t="inlineStr">
+        <is>
+          <t>EMS.QA.FRM.03.05</t>
+        </is>
       </c>
       <c r="AR2" s="24"/>
       <c r="AS2" s="24"/>
@@ -6704,8 +6706,10 @@
       <c r="AN2" s="23"/>
       <c r="AO2" s="23"/>
       <c r="AP2" s="23"/>
-      <c r="AQ2" s="24" t="s">
-        <v>46</v>
+      <c r="AQ2" s="24" t="inlineStr">
+        <is>
+          <t>EMS.QA.FRM.03.05</t>
+        </is>
       </c>
       <c r="AR2" s="24"/>
       <c r="AS2" s="24"/>

</xml_diff>

<commit_message>
İki formun iç belge numarası dosya koduyla eşitlendi; belge senkron raporu ve içerik kontrolü notu (#473)
Claude-Session: https://claude.ai/code/session_01J6foNXTwf1dGzDjULYpfrk

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/formlar/4. Dikimhane Bölümü/EMS.QA.FRM.03.05. QA_Baskı Nakış Onay Formu.xlsx
+++ b/formlar/4. Dikimhane Bölümü/EMS.QA.FRM.03.05. QA_Baskı Nakış Onay Formu.xlsx
@@ -4897,8 +4897,10 @@
       <c r="AN2" s="87"/>
       <c r="AO2" s="87"/>
       <c r="AP2" s="87"/>
-      <c r="AQ2" s="24" t="s">
-        <v>46</v>
+      <c r="AQ2" s="24" t="inlineStr">
+        <is>
+          <t>EMS.QA.FRM.03.05</t>
+        </is>
       </c>
       <c r="AR2" s="24"/>
       <c r="AS2" s="24"/>
@@ -6704,8 +6706,10 @@
       <c r="AN2" s="23"/>
       <c r="AO2" s="23"/>
       <c r="AP2" s="23"/>
-      <c r="AQ2" s="24" t="s">
-        <v>46</v>
+      <c r="AQ2" s="24" t="inlineStr">
+        <is>
+          <t>EMS.QA.FRM.03.05</t>
+        </is>
       </c>
       <c r="AR2" s="24"/>
       <c r="AS2" s="24"/>

</xml_diff>